<commit_message>
Update ransomware news feed
</commit_message>
<xml_diff>
--- a/data/latest_ransomware_news.xlsx
+++ b/data/latest_ransomware_news.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -898,6 +898,105 @@
         <v>46011.59137731481</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Qilin</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>"Qilin ransomware" OR "Qilin threat actor" OR "Qilin cyber attack"</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Nissan confirms data compromise from Red Hat hack - SC Media</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 18:19:11 GMT</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxNLXR1V3lEZjBrd2h0TWF4REozNU83M2o5bUUxemY2eWh1Y3RQTngwYzktbW1JakpvdnN5NG10aGl1SG5zcjNSMG9TUWxMemJDWE9MTENyMG44aUlqbmNBVndZZHl2S2Rtbkh1d2l6NEdIcGxtLV9PaTMzTm9NbTd2OS1DdFMwUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>7</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>46014.76332175926</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Medusa</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>"Medusa ransomware" OR "Medusa threat actor" OR "Medusa cyber attack"</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>WordPress plugin auth bypass exploited almost immediately after disclosure - MSN</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 15:59:23 GMT</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9wJBVV95cUxOMldFd3JmaVBiM2lmSnNtMFhjOHRFUDZzVTdWd0hhSFZNMkR5a19hTEFIeEExUGZWcTRuTHNtXzdSbUJ2MVJxSzZhd0ZxVHBtUTRUTzZualVpQ2xUdzRQdWpFNndDZm4wd1dnWXZ3WUkwYi1tSVNuaWd2REdRbkthdUpXdjJadzNpVmNscE9ITTZlaFhHZVg1Y1dYbHNUUHNLb2NKQU9uME1Wd2w1bm1kR3NMSHJRUkhkUVBSR1B2QlJfVEF6UVZfUlJ3NjBuR1gxaVVONUQybEpKQy16bWFxcFJQR0dMbENnZzNoZVRuMzU2NHFCX1lBeU04WDV2WDBrZ2lROV81OVd5ZDZsemk2MEdHZUhiOG1GUUdvT0N1LTdRc2gxRWk4c3FzVkgyczNrT2s4NV91X1FaMEp1RmtDdC00YTRQaENlNjZ3ZnRuak81Mk5JZGEwWFY5Zzh6YkFpUVZFejV3M3d0Y3NvYko3WmtlUTBmNG8?oc=5</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>7</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>46014.66623842593</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Medusa</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>"Medusa ransomware" OR "Medusa threat actor" OR "Medusa cyber attack"</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CISA loses key employee behind early ransomware warnings - itsecuritynews.info</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Tue, 23 Dec 2025 16:02:53 GMT</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQYnNvUnJieV9TaVdiSEFzRTJobUxaam1XOG82d3lZRktPSEJnWVhRNlY0VEJ0Q25QMi16bzhHa0NIX0FKNWRrVXUteTZGeXJ1NmItNHhfN1FxeHEyNkNNYzdDb2pVcG14VXEwc25hNU84Zm5iN1VDcTNTTkltUEZXdU5aZEVab2NYaVl5QnpraTk5R0k?oc=5</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>7</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>46014.66866898148</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>